<commit_message>
feat(data): sintetik tanlanmani rasmiy agregat statistikaga moslashtirish
- Hududlar ulushi: faoliyat ko'rsatayotgan korxonalar soni (2026-04-01, 577,2 ming)
- Sohalar ulushi: faoliyat turlari bo'yicha korxonalar soni (2026-08-01, 601,3 ming)
- Soha o'rtacha oylik aylanmasi: 2025-yil hajmi / korxonalar soni / 12
  (sanoat 1 101,1; qurilish 313,9; chakana savdo 482,4; qishloq xo'jaligi 538,9;
  bozor xizmatlari 1 050,3 trln so'm), post-stratifikatsiya bilan ±2% aniqlikda
- Hududiy daraja 2025-yil YaHM asosida; kichik korxonalar ulushi 84,9%
- Sohalar rasmiy tasnifga keltirildi (10 ta); ta'lim olib tashlandi (umumiy son topilmadi)
- Manbalar, taxminlar va tanlanma/rasmiy taqqoslash: /data-sources/calibration va UI paneli
- Xavf baholari o'zgarmadi (nisbiy belgilar); 2 ta yangi test (jami 42)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/samples/namuna_tranzaksiyalar.xlsx
+++ b/data/samples/namuna_tranzaksiyalar.xlsx
@@ -458,7 +458,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>969306635</t>
+          <t>903392201</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -479,7 +479,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>959505164</t>
+          <t>967603782</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -500,7 +500,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>967603782</t>
+          <t>955840825</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -521,7 +521,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>955840825</t>
+          <t>976555774</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -542,7 +542,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>976555774</t>
+          <t>928375954</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -563,7 +563,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>928375954</t>
+          <t>990695810</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -584,7 +584,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>918332710</t>
+          <t>915283110</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -605,7 +605,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>963986608</t>
+          <t>978083008</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -626,7 +626,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>900619063</t>
+          <t>985937489</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -647,7 +647,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>915283110</t>
+          <t>903705377</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -668,7 +668,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>978083008</t>
+          <t>901456310</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -689,7 +689,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>985937489</t>
+          <t>908780916</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -710,7 +710,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>901456310</t>
+          <t>992750649</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -731,7 +731,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>933129848</t>
+          <t>938962454</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -752,7 +752,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>938962454</t>
+          <t>974244224</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -773,7 +773,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>942520740</t>
+          <t>944640369</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -794,7 +794,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>959024829</t>
+          <t>907910892</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -815,7 +815,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>988553320</t>
+          <t>974424931</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -857,7 +857,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>970221388</t>
+          <t>906596525</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -878,7 +878,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>985986908</t>
+          <t>970221388</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -899,7 +899,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>917813720</t>
+          <t>985986908</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -962,7 +962,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>916580374</t>
+          <t>946813044</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>946813044</t>
+          <t>978887439</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1004,7 +1004,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>978887439</t>
+          <t>925527658</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1025,7 +1025,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>996782733</t>
+          <t>954942204</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1046,7 +1046,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>925527658</t>
+          <t>974611290</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1067,7 +1067,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>979927823</t>
+          <t>916795388</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1088,7 +1088,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>984095398</t>
+          <t>965533161</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1109,7 +1109,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>954942204</t>
+          <t>992041186</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1130,7 +1130,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>956405127</t>
+          <t>960771222</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1151,7 +1151,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>906870564</t>
+          <t>998727787</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1172,7 +1172,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>957168017</t>
+          <t>909520378</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1193,7 +1193,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>965533161</t>
+          <t>910972242</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1214,7 +1214,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>954959330</t>
+          <t>946076843</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1235,7 +1235,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>998727787</t>
+          <t>900316300</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1256,7 +1256,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>925305248</t>
+          <t>937705653</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1277,7 +1277,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>909520378</t>
+          <t>955490517</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1298,7 +1298,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>955840825</t>
+          <t>976555774</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1340,7 +1340,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>963986608</t>
+          <t>978083008</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1361,7 +1361,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>915283110</t>
+          <t>903705377</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1382,7 +1382,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>985937489</t>
+          <t>908780916</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">

</xml_diff>